<commit_message>
Add lifecycle walkthrough notebook and full README
Notebook walks the full engagement financial lifecycle end-to-end in the
voice of an engagement finance associate, from portfolio setup through
the discrepancy exception report -- executed cleanly with real outputs
cached. README explains what engagement/account finance operations means
in a professional-services context, what each control catches and why,
how to run the toolkit, and the synthetic-data disclaimer.

Also regenerates the committed sample workbook from the latest pipeline
run (recalculated, zero formula errors).
</commit_message>
<xml_diff>
--- a/output/engagement_finance_toolkit.xlsx
+++ b/output/engagement_finance_toolkit.xlsx
@@ -1570,11 +1570,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="90266516"/>
-        <c:axId val="10952827"/>
+        <c:axId val="86322139"/>
+        <c:axId val="60669824"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="90266516"/>
+        <c:axId val="86322139"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1640,7 +1640,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="10952827"/>
+        <c:crossAx val="60669824"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1648,7 +1648,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="10952827"/>
+        <c:axId val="60669824"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1724,7 +1724,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="90266516"/>
+        <c:crossAx val="86322139"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2104,11 +2104,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="10060181"/>
-        <c:axId val="26986351"/>
+        <c:axId val="69944709"/>
+        <c:axId val="66833694"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="10060181"/>
+        <c:axId val="69944709"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2174,7 +2174,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="26986351"/>
+        <c:crossAx val="66833694"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2182,7 +2182,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="26986351"/>
+        <c:axId val="66833694"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2258,7 +2258,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="10060181"/>
+        <c:crossAx val="69944709"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2441,11 +2441,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="86867025"/>
-        <c:axId val="1212744"/>
+        <c:axId val="40199821"/>
+        <c:axId val="3477058"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="86867025"/>
+        <c:axId val="40199821"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2477,7 +2477,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1212744"/>
+        <c:crossAx val="3477058"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2485,7 +2485,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1212744"/>
+        <c:axId val="3477058"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2561,7 +2561,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86867025"/>
+        <c:crossAx val="40199821"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>

<commit_message>
Refresh sample workbook from latest verified pipeline run
Regenerated and recalculated (1,271 formulas, 0 errors) while pulling
verified output numbers for resume/interview talking points. Same
deterministic seed, no logic changes.
</commit_message>
<xml_diff>
--- a/output/engagement_finance_toolkit.xlsx
+++ b/output/engagement_finance_toolkit.xlsx
@@ -1570,11 +1570,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="86322139"/>
-        <c:axId val="60669824"/>
+        <c:axId val="51774081"/>
+        <c:axId val="47281745"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="86322139"/>
+        <c:axId val="51774081"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1640,7 +1640,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60669824"/>
+        <c:crossAx val="47281745"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1648,7 +1648,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="60669824"/>
+        <c:axId val="47281745"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1724,7 +1724,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86322139"/>
+        <c:crossAx val="51774081"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2104,11 +2104,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="69944709"/>
-        <c:axId val="66833694"/>
+        <c:axId val="84332220"/>
+        <c:axId val="96267404"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="69944709"/>
+        <c:axId val="84332220"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2174,7 +2174,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="66833694"/>
+        <c:crossAx val="96267404"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2182,7 +2182,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="66833694"/>
+        <c:axId val="96267404"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2258,7 +2258,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="69944709"/>
+        <c:crossAx val="84332220"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2441,11 +2441,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="40199821"/>
-        <c:axId val="3477058"/>
+        <c:axId val="20629070"/>
+        <c:axId val="18265195"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="40199821"/>
+        <c:axId val="20629070"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2477,7 +2477,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="3477058"/>
+        <c:crossAx val="18265195"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2485,7 +2485,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="3477058"/>
+        <c:axId val="18265195"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2561,7 +2561,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40199821"/>
+        <c:crossAx val="20629070"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>